<commit_message>
updated with crew suggestion
</commit_message>
<xml_diff>
--- a/llm_usage_log.xlsx
+++ b/llm_usage_log.xlsx
@@ -421,7 +421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -729,26 +729,229 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2">
-        <f>"TOTAL calls: "&amp;COUNTA(A2:A10)</f>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-09-16T10:48:49+00:00</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>gpt-4o-mini</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>3.475</v>
+      </c>
+      <c r="E11" t="n">
+        <v>3385</v>
+      </c>
+      <c r="F11" t="n">
+        <v>333</v>
+      </c>
+      <c r="G11" t="n">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-09-16T10:49:12+00:00</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>gpt-4o-mini</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>2.663</v>
+      </c>
+      <c r="E12" t="n">
+        <v>3964</v>
+      </c>
+      <c r="F12" t="n">
+        <v>255</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-09-16T10:49:27+00:00</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>gpt-4o-mini</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>2.378</v>
+      </c>
+      <c r="E13" t="n">
+        <v>1819</v>
+      </c>
+      <c r="F13" t="n">
+        <v>236</v>
+      </c>
+      <c r="G13" t="n">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-09-16T10:51:59+00:00</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>gpt-4o-mini</t>
+        </is>
+      </c>
+      <c r="D14" t="n">
+        <v>3.101</v>
+      </c>
+      <c r="E14" t="n">
+        <v>1810</v>
+      </c>
+      <c r="F14" t="n">
+        <v>247</v>
+      </c>
+      <c r="G14" t="n">
+        <v>1024</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-09-17T04:52:27+00:00</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>gpt-4o-mini</t>
+        </is>
+      </c>
+      <c r="D15" t="n">
+        <v>3.949</v>
+      </c>
+      <c r="E15" t="n">
+        <v>2645</v>
+      </c>
+      <c r="F15" t="n">
+        <v>261</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-09-17T04:56:23+00:00</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>gpt-4o-mini</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>2.576</v>
+      </c>
+      <c r="E16" t="n">
+        <v>2658</v>
+      </c>
+      <c r="F16" t="n">
+        <v>245</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-09-17T04:58:08+00:00</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>openai</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>gpt-4o-mini</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>2.855</v>
+      </c>
+      <c r="E17" t="n">
+        <v>2664</v>
+      </c>
+      <c r="F17" t="n">
+        <v>253</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2176</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2">
+        <f>"TOTAL calls: "&amp;COUNTA(A2:A17)</f>
         <v/>
       </c>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2">
-        <f>SUM(D2:D10)</f>
+      <c r="B18" s="2" t="n"/>
+      <c r="C18" s="2" t="n"/>
+      <c r="D18" s="2">
+        <f>SUM(D2:D17)</f>
         <v/>
       </c>
-      <c r="E11" s="2">
-        <f>SUM(E2:E10)</f>
+      <c r="E18" s="2">
+        <f>SUM(E2:E17)</f>
         <v/>
       </c>
-      <c r="F11" s="2">
-        <f>SUM(F2:F10)</f>
+      <c r="F18" s="2">
+        <f>SUM(F2:F17)</f>
         <v/>
       </c>
-      <c r="G11" s="2">
-        <f>SUM(G2:G10)</f>
+      <c r="G18" s="2">
+        <f>SUM(G2:G17)</f>
         <v/>
       </c>
     </row>

</xml_diff>